<commit_message>
Add #555 wedge LED lamp bulbs + sockets to the BOM
The 16 score lamps (10-400 + Winner/Game Over/Tilt) and their sockets
were missing. Added #555 T10 wedge LED bulbs (6.3 V, non-polar, built-in
resistor) and pigtail wedge sockets to the sourced BOM, the schematic-page
BOM image, and the assembly guide. BOM total is now $473.52.
</commit_message>
<xml_diff>
--- a/docs/SkillGame BOM (sourced).xlsx
+++ b/docs/SkillGame BOM (sourced).xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1215,37 +1215,37 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Actuators</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Coin-Lock, Win-Lock</t>
+          <t>Score lamps</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>SparkFun Solenoid - 5V (Small)</t>
+          <t>#555 T10 wedge LED, 6.3V non-polar (frosted)</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>20-pack</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>SparkFun ROB-11015</t>
+          <t>Amazon (Keiurot)</t>
         </is>
       </c>
       <c r="G19" s="12" t="n">
-        <v>4.95</v>
+        <v>16</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>9.9</v>
+        <v>16</v>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
@@ -1254,44 +1254,74 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>small 5 V coils, ~4.5 mm throw</t>
+          <t>16 lamps (10-400 + Winner/GO/Tilt); built-in resistor — on 5V + the board's 220R they run dim, jumper the 220R or feed 6.3V for full brightness</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Lamp sockets</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>T10/#555 wedge socket, pigtail leads</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>20-pack</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Amazon B00VDOPPDE</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>pre-wired; solder to the J2 lamp lines</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>mini-PC</t>
+          <t>Coin-Lock, Win-Lock</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>PELADN Ryzen 5 5600H, 16GB DDR4 / 512GB SSD</t>
+          <t>SparkFun Solenoid - 5V (Small)</t>
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
@@ -1300,14 +1330,14 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Amazon B0F7R7V9VK</t>
+          <t>SparkFun ROB-11015</t>
         </is>
       </c>
       <c r="G21" s="12" t="n">
-        <v>209.99</v>
+        <v>4.95</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>209.99</v>
+        <v>9.9</v>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
@@ -1316,70 +1346,40 @@
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>6C/12T Ryzen, Vega gfx, WiFi6, USB3.2 — plenty of headroom</t>
+          <t>small 5 V coils, ~4.5 mm throw</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>QQU 15.6" portable touchscreen (with stand)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Amazon B0FHHM1Y7Z</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>70.48999999999999</v>
-      </c>
-      <c r="H22" s="8" t="n">
-        <v>70.48999999999999</v>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>1080P IPS/HDR; USB-C touch + HDMI; incl. stand</t>
-        </is>
-      </c>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>mini-PC</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>4-port USB 2.0 hub</t>
+          <t>PELADN Ryzen 5 5600H, 16GB DDR4 / 512GB SSD</t>
         </is>
       </c>
       <c r="D23" s="10" t="n">
@@ -1392,14 +1392,14 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Amazon/Monoprice</t>
+          <t>Amazon B0F7R7V9VK</t>
         </is>
       </c>
       <c r="G23" s="12" t="n">
-        <v>8.99</v>
+        <v>209.99</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>8.99</v>
+        <v>209.99</v>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
@@ -1408,24 +1408,24 @@
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>one port per FT232H</t>
+          <t>6C/12T Ryzen, Vega gfx, WiFi6, USB3.2 — plenty of headroom</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Display</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>J1 supply</t>
+          <t>monitor</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>3.3 V DC wall adapter (≥1A)</t>
+          <t>QQU 15.6" portable touchscreen (with stand)</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
@@ -1438,14 +1438,14 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Amazon B07BGW2VXV</t>
+          <t>Amazon B0FHHM1Y7Z</t>
         </is>
       </c>
       <c r="G24" s="8" t="n">
-        <v>7.99</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>7.99</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
@@ -1454,24 +1454,24 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>switch-common / GPIO logic</t>
+          <t>1080P IPS/HDR; USB-C touch + HDMI; incl. stand</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>J3 / LED± supply</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>5 V DC wall adapter (≥5A)</t>
+          <t>4-port USB 2.0 hub</t>
         </is>
       </c>
       <c r="D25" s="10" t="n">
@@ -1484,39 +1484,131 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
+          <t>Amazon/Monoprice</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>one port per FT232H</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>J1 supply</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>3.3 V DC wall adapter (≥1A)</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Amazon B07BGW2VXV</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>switch-common / GPIO logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>J3 / LED± supply</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>5 V DC wall adapter (≥5A)</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
           <t>Amazon (5V 5A)</t>
         </is>
       </c>
-      <c r="G25" s="12" t="n">
+      <c r="G27" s="12" t="n">
         <v>12.99</v>
       </c>
-      <c r="H25" s="12" t="n">
+      <c r="H27" s="12" t="n">
         <v>12.99</v>
       </c>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J25" s="11" t="inlineStr">
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
         <is>
           <t>size for LED strip + lamps + coils</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="G27" s="14" t="inlineStr">
+    <row r="29">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>ESTIMATED TOTAL</t>
         </is>
       </c>
-      <c r="H27" s="15">
-        <f>SUM(H5:H25)</f>
+      <c r="H29" s="15">
+        <f>SUM(H5:H27)</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="C28" s="16" t="inlineStr">
+    <row r="30">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>Line est already accounts for quantity (e.g. 4× FT232H). Pack/kit rows are a single purchase that covers the qty.</t>
         </is>
@@ -1524,9 +1616,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A22:J22"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A20:J20"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <hyperlinks>
@@ -1544,11 +1636,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show the LED lamps in the schematic; double the 100/200/300/400 holes
- Schematic: added all 16 score-lamp bulbs as #555 wedge LED symbols, with
  the 100/200/300/400 holes drawing TWO bulbs each (parallel, same output)
  for double brightness. Non-polar bulbs; ERC clean.
- The board's lamp resistors R30-R62 are now 0 R links (schematic + PCB) --
  the pre-resistored #555 bulb self-limits and a 6.3 V bulb is safely
  under-driven on the 5 V rail. DRC clean.
- App: the SCORE LAMPS block now shows the LED bulb bank; updated the lamp
  and 5 V-rail text to match (no more 220 ohm).
- BOM + assembly guide: 20 #555 bulbs + 20 sockets, 0 R lamp links, and the
  WezeBull logo on the guide's cover. Sourced BOM total now $477.52.
- README: logo, badges, How-it-plays, Features and Hardware sections.
</commit_message>
<xml_diff>
--- a/docs/SkillGame BOM (sourced).xlsx
+++ b/docs/SkillGame BOM (sourced).xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -806,16 +806,16 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>R1–R62</t>
+          <t>R1–R29 + bases</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>1/4 W resistor assortment (10k/1k/220/2.2k)</t>
+          <t>1/4 W resistor assortment (10k/1k/2.2k)</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -840,28 +840,28 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>28×10k, 16×1k, 16×220, 2×2.2k — kit covers all</t>
+          <t>28×10k pull-downs, 16×1k bases, 2×2.2k TIP120 bases (kit covers all)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>Jumpers</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>F1, F2</t>
+          <t>R30–R62</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Littelfuse 0218002.MXP T2A 5×20mm 250V</t>
+          <t>0 Ω lamp links (bridge with wire / solder)</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
@@ -870,14 +870,14 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>DigiKey 777600</t>
+          <t>in kit / solder</t>
         </is>
       </c>
       <c r="G11" s="12" t="n">
-        <v>0.68</v>
+        <v>0</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>1.36</v>
+        <v>0</v>
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>slow-blow; for the small 5V solenoids</t>
+          <t>lamp positions — the #555 bulb self-limits, so these are 0 Ω links, not resistors</t>
         </is>
       </c>
     </row>
@@ -898,16 +898,16 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F1, F2</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Bussmann GDC-3.5A T3.5A 5×20mm 250V</t>
+          <t>Littelfuse 0218002.MXP T2A 5×20mm 250V</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
@@ -916,14 +916,14 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>DigiKey/Mouser</t>
+          <t>DigiKey 777600</t>
         </is>
       </c>
       <c r="G12" s="8" t="n">
-        <v>1.1</v>
+        <v>0.68</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>1.1</v>
+        <v>1.36</v>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>inline main fuse in the 5V lead to J3</t>
+          <t>slow-blow; for the small 5V solenoids</t>
         </is>
       </c>
     </row>
@@ -944,16 +944,16 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>F1, F2 holders</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Keystone 3517 fuse clip 5×20mm</t>
+          <t>Bussmann GDC-3.5A T3.5A 5×20mm 250V</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
@@ -962,14 +962,14 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>DigiKey 316010</t>
+          <t>DigiKey/Mouser</t>
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>0.3</v>
+        <v>1.1</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>2 clips per fuse (F1/F2)</t>
+          <t>inline main fuse in the 5V lead to J3</t>
         </is>
       </c>
     </row>
@@ -990,16 +990,16 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>F3 holder</t>
+          <t>F1, F2 holders</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Inline 5×20mm fuse holder (in-lead)</t>
+          <t>Keystone 3517 fuse clip 5×20mm</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
@@ -1008,14 +1008,14 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Amazon/DigiKey</t>
+          <t>DigiKey 316010</t>
         </is>
       </c>
       <c r="G14" s="8" t="n">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
@@ -1024,24 +1024,24 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>holds F3 in the 5 V supply wire</t>
+          <t>2 clips per fuse (F1/F2)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Connectors</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>F3 holder</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>2×20 (40-pin) 2.54mm header</t>
+          <t>Inline 5×20mm fuse holder (in-lead)</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
@@ -1054,14 +1054,14 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>Amazon/DigiKey</t>
         </is>
       </c>
       <c r="G15" s="12" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>lamp/output connector</t>
+          <t>holds F3 in the 5 V supply wire</t>
         </is>
       </c>
     </row>
@@ -1082,20 +1082,20 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>J1,J3,J4,J5</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>2-pin 2.54mm header</t>
+          <t>2×20 (40-pin) 2.54mm header</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>each</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1104,10 +1104,10 @@
         </is>
       </c>
       <c r="G16" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
@@ -1116,44 +1116,44 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>power in + solenoid out</t>
+          <t>lamp/output connector</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Playfield</t>
+          <t>Connectors</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>SW0–SW27 (+SW23×7)</t>
+          <t>J1,J3,J4,J5</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Leaf / micro switches</t>
+          <t>2-pin 2.54mm header</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>source to fit</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="G17" s="12" t="n">
-        <v>0.45</v>
+        <v>3</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>15.3</v>
+        <v>3</v>
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
@@ -1162,28 +1162,28 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>28 logical inputs; reuse originals if possible</t>
+          <t>power in + solenoid out</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Playfield</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>LED strip</t>
+          <t>SW0–SW27 (+SW23×7)</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>WS2812b 150-pixel 5V strip</t>
+          <t>Leaf / micro switches</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
@@ -1192,14 +1192,14 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Amazon B0CFTPT81S</t>
+          <t>source to fit</t>
         </is>
       </c>
       <c r="G18" s="8" t="n">
-        <v>12.99</v>
+        <v>0.45</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>12.99</v>
+        <v>15.3</v>
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>150 addressable px</t>
+          <t>28 logical inputs; reuse originals if possible</t>
         </is>
       </c>
     </row>
@@ -1220,32 +1220,32 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Score lamps</t>
+          <t>LED strip</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>#555 T10 wedge LED, 6.3V non-polar (frosted)</t>
+          <t>WS2812b 150-pixel 5V strip</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>20-pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Amazon (Keiurot)</t>
+          <t>Amazon B0CFTPT81S</t>
         </is>
       </c>
       <c r="G19" s="12" t="n">
-        <v>16</v>
+        <v>12.99</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>16</v>
+        <v>12.99</v>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>16 lamps (10-400 + Winner/GO/Tilt); built-in resistor — on 5V + the board's 220R they run dim, jumper the 220R or feed 6.3V for full brightness</t>
+          <t>150 addressable px</t>
         </is>
       </c>
     </row>
@@ -1266,32 +1266,32 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Lamp sockets</t>
+          <t>Score lamps</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>T10/#555 wedge socket, pigtail leads</t>
+          <t>#555 T10 wedge LED, 6.3V non-polar (frosted)</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>20-pack</t>
+          <t>25-pack</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Amazon B00VDOPPDE</t>
+          <t>Amazon (Keiurot)</t>
         </is>
       </c>
       <c r="G20" s="8" t="n">
-        <v>9.99</v>
+        <v>18</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>9.99</v>
+        <v>18</v>
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
@@ -1300,132 +1300,132 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>pre-wired; solder to the J2 lamp lines</t>
+          <t>16 lamps + a 2nd bulb on 100/200/300/400 (double bright) = 20; non-polar &amp; pre-resistored, runs safely under-driven on the 5V rail (board R = 0 ohm links)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Lamp sockets</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>T10/#555 wedge socket, pigtail leads</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>25-pack</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Amazon B00VDOPPDE</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>one per bulb; solder its leads to the J2 lamp lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>Actuators</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Coin-Lock, Win-Lock</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>SparkFun Solenoid - 5V (Small)</t>
         </is>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D22" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>each</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>SparkFun ROB-11015</t>
         </is>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="G22" s="8" t="n">
         <v>4.95</v>
       </c>
-      <c r="H21" s="12" t="n">
+      <c r="H22" s="8" t="n">
         <v>9.9</v>
       </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J21" s="11" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>small 5 V coils, ~4.5 mm throw</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="5" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>Computer</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>mini-PC</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>PELADN Ryzen 5 5600H, 16GB DDR4 / 512GB SSD</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Amazon B0F7R7V9VK</t>
-        </is>
-      </c>
-      <c r="G23" s="12" t="n">
-        <v>209.99</v>
-      </c>
-      <c r="H23" s="12" t="n">
-        <v>209.99</v>
-      </c>
-      <c r="I23" s="13" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J23" s="11" t="inlineStr">
-        <is>
-          <t>6C/12T Ryzen, Vega gfx, WiFi6, USB3.2 — plenty of headroom</t>
-        </is>
-      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Display</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>monitor</t>
+          <t>mini-PC</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>QQU 15.6" portable touchscreen (with stand)</t>
+          <t>PELADN Ryzen 5 5600H, 16GB DDR4 / 512GB SSD</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
@@ -1438,14 +1438,14 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Amazon B0FHHM1Y7Z</t>
+          <t>Amazon B0F7R7V9VK</t>
         </is>
       </c>
       <c r="G24" s="8" t="n">
-        <v>70.48999999999999</v>
+        <v>209.99</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>70.48999999999999</v>
+        <v>209.99</v>
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
@@ -1454,24 +1454,24 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>1080P IPS/HDR; USB-C touch + HDMI; incl. stand</t>
+          <t>6C/12T Ryzen, Vega gfx, WiFi6, USB3.2 — plenty of headroom</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>Display</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>monitor</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>4-port USB 2.0 hub</t>
+          <t>QQU 15.6" portable touchscreen (with stand)</t>
         </is>
       </c>
       <c r="D25" s="10" t="n">
@@ -1484,14 +1484,14 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Amazon/Monoprice</t>
+          <t>Amazon B0FHHM1Y7Z</t>
         </is>
       </c>
       <c r="G25" s="12" t="n">
-        <v>8.99</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>8.99</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
@@ -1500,24 +1500,24 @@
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>one port per FT232H</t>
+          <t>1080P IPS/HDR; USB-C touch + HDMI; incl. stand</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>J1 supply</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>3.3 V DC wall adapter (≥1A)</t>
+          <t>4-port USB 2.0 hub</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
@@ -1530,14 +1530,14 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Amazon B07BGW2VXV</t>
+          <t>Amazon/Monoprice</t>
         </is>
       </c>
       <c r="G26" s="8" t="n">
-        <v>7.99</v>
+        <v>8.99</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>7.99</v>
+        <v>8.99</v>
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>switch-common / GPIO logic</t>
+          <t>one port per FT232H</t>
         </is>
       </c>
     </row>
@@ -1558,12 +1558,12 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>J3 / LED± supply</t>
+          <t>J1 supply</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>5 V DC wall adapter (≥5A)</t>
+          <t>3.3 V DC wall adapter (≥1A)</t>
         </is>
       </c>
       <c r="D27" s="10" t="n">
@@ -1576,39 +1576,85 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
+          <t>Amazon B07BGW2VXV</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>switch-common / GPIO logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>J3 / LED± supply</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>5 V DC wall adapter (≥5A)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
           <t>Amazon (5V 5A)</t>
         </is>
       </c>
-      <c r="G27" s="12" t="n">
+      <c r="G28" s="8" t="n">
         <v>12.99</v>
       </c>
-      <c r="H27" s="12" t="n">
+      <c r="H28" s="8" t="n">
         <v>12.99</v>
       </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J27" s="11" t="inlineStr">
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>size for LED strip + lamps + coils</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="G29" s="14" t="inlineStr">
+    <row r="30">
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>ESTIMATED TOTAL</t>
         </is>
       </c>
-      <c r="H29" s="15">
-        <f>SUM(H5:H27)</f>
+      <c r="H30" s="15">
+        <f>SUM(H5:H28)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="C30" s="16" t="inlineStr">
+    <row r="31">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>Line est already accounts for quantity (e.g. 4× FT232H). Pack/kit rows are a single purchase that covers the qty.</t>
         </is>
@@ -1616,7 +1662,7 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="A2:J2"/>
@@ -1638,11 +1684,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add wiring harnesses, playfield maps, F3 cable, and switch sourcing
- Wiring harnesses for the lamps and switches: flat diagrams with every
  solder point, 3D cable views, and playfield/backglass maps showing where
  each lamp socket and switch lands (switch positions traced from the real
  Skill-Roll board).
- Inline fuse cable (F3): dedicated diagram + 3D view; pinned the holder to
  a real part (uxcell 18 AWG inline, B07SM5KYZ7).
- Score-lamp doubling (100/200/300/400) and 0 R lamp-link detail added to
  the guide with diagrams.
- Switches: the Bally rollover-wire switch is discontinued -- recommend a
  mini hinge-lever microswitch (in stock) with the Action Pinball SW-1A-120
  as the authentic alternative.
- Guide expanded to 23 pages (more detail per step, WezeBull logo cover).
  Sourced BOM total now $499.67.
</commit_message>
<xml_diff>
--- a/docs/SkillGame BOM (sourced).xlsx
+++ b/docs/SkillGame BOM (sourced).xlsx
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Inline 5×20mm fuse holder (in-lead)</t>
+          <t>uxcell inline screw-type 5×20mm fuse holder, 18 AWG leads</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>5-pack</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Amazon/DigiKey</t>
+          <t>Amazon B07SM5KYZ7</t>
         </is>
       </c>
       <c r="G15" s="12" t="n">
-        <v>1.5</v>
+        <v>6.99</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>1.5</v>
+        <v>6.99</v>
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>holds F3 in the 5 V supply wire</t>
+          <t>splices into the 5 V supply wire feeding J3; 18 AWG handles the 3.5 A rail</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1174,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>SW0–SW27 (+SW23×7)</t>
+          <t>Score / gobble switches</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Leaf / micro switches</t>
+          <t>Mini snap-action microswitch, hinge/roller lever (SPDT)</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -1187,19 +1187,19 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>4x10-pack</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>source to fit</t>
+          <t>Amazon B0C6ZNBFDH</t>
         </is>
       </c>
       <c r="G18" s="8" t="n">
-        <v>0.45</v>
+        <v>31.96</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>15.3</v>
+        <v>31.96</v>
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>28 logical inputs; reuse originals if possible</t>
+          <t>lever pokes up through the playfield slot, the coin trips it (28 inputs; the 7 gobble switches parallel onto S23). Authentic alt: the Bally rollover-wire leaf switch is DISCONTINUED - Action Pinball SW-1A-120 ($8.39 ea, in stock) needs a rollover wireform. Reuse your originals if you have them.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 28 switch-input debounce caps (100 nF) to the board
- Schematic: added C1-C28, one 100 nF cap from each switch input to GND,
  in parallel with the 10k pull-down (~1 ms RC debounce + noise filter on
  the long playfield leads). Enlarged the sheet to fit the cap bank. ERC at
  the benign baseline; all 28 netlist-verified across input<->GND.
- PCB: placed all 28 as 0805 SMD on the back, next to each pull-down (GND
  pad on the pour, input to the pull-down). 3D back render updated.
- BOM + guide + app schematic images updated (BOM total now $507.16, guide
  24 pages with a debounce-cap step). Synced to the live OneDrive KiCad.
</commit_message>
<xml_diff>
--- a/docs/SkillGame BOM (sourced).xlsx
+++ b/docs/SkillGame BOM (sourced).xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -893,37 +893,37 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>Filtering</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>F1, F2</t>
+          <t>C1–C28</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Littelfuse 0218002.MXP T2A 5×20mm 250V</t>
+          <t>0.1 uF (100 nF) ceramic cap, 0805 SMD</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>50-pack</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>DigiKey 777600</t>
+          <t>Amazon (100nF 0805)</t>
         </is>
       </c>
       <c r="G12" s="8" t="n">
-        <v>0.68</v>
+        <v>7.49</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>1.36</v>
+        <v>7.49</v>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>slow-blow; for the small 5V solenoids</t>
+          <t>one per switch input to GND — debounce + noise filter (~1 ms RC with the 10k pull-down); on the board's back side</t>
         </is>
       </c>
     </row>
@@ -944,16 +944,16 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F1, F2</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Bussmann GDC-3.5A T3.5A 5×20mm 250V</t>
+          <t>Littelfuse 0218002.MXP T2A 5×20mm 250V</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
@@ -962,14 +962,14 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>DigiKey/Mouser</t>
+          <t>DigiKey 777600</t>
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>1.1</v>
+        <v>0.68</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>1.1</v>
+        <v>1.36</v>
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>inline main fuse in the 5V lead to J3</t>
+          <t>slow-blow; for the small 5V solenoids</t>
         </is>
       </c>
     </row>
@@ -990,16 +990,16 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>F1, F2 holders</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Keystone 3517 fuse clip 5×20mm</t>
+          <t>Bussmann GDC-3.5A T3.5A 5×20mm 250V</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
@@ -1008,14 +1008,14 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>DigiKey 316010</t>
+          <t>DigiKey/Mouser</t>
         </is>
       </c>
       <c r="G14" s="8" t="n">
-        <v>0.3</v>
+        <v>1.1</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>2 clips per fuse (F1/F2)</t>
+          <t>inline main fuse in the 5V lead to J3</t>
         </is>
       </c>
     </row>
@@ -1036,32 +1036,32 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>F3 holder</t>
+          <t>F1, F2 holders</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>uxcell inline screw-type 5×20mm fuse holder, 18 AWG leads</t>
+          <t>Keystone 3517 fuse clip 5×20mm</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>5-pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Amazon B07SM5KYZ7</t>
+          <t>DigiKey 316010</t>
         </is>
       </c>
       <c r="G15" s="12" t="n">
-        <v>6.99</v>
+        <v>0.3</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>6.99</v>
+        <v>1.2</v>
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
@@ -1070,24 +1070,24 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>splices into the 5 V supply wire feeding J3; 18 AWG handles the 3.5 A rail</t>
+          <t>2 clips per fuse (F1/F2)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Connectors</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>F3 holder</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>2×20 (40-pin) 2.54mm header</t>
+          <t>uxcell inline screw-type 5×20mm fuse holder, 18 AWG leads</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>5-pack</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>Amazon B07SM5KYZ7</t>
         </is>
       </c>
       <c r="G16" s="8" t="n">
-        <v>1</v>
+        <v>6.99</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>1</v>
+        <v>6.99</v>
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>lamp/output connector</t>
+          <t>splices into the 5 V supply wire feeding J3; 18 AWG handles the 3.5 A rail</t>
         </is>
       </c>
     </row>
@@ -1128,20 +1128,20 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>J1,J3,J4,J5</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>2-pin 2.54mm header</t>
+          <t>2×20 (40-pin) 2.54mm header</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>each</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
@@ -1150,10 +1150,10 @@
         </is>
       </c>
       <c r="G17" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
@@ -1162,44 +1162,44 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>power in + solenoid out</t>
+          <t>lamp/output connector</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Playfield</t>
+          <t>Connectors</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Score / gobble switches</t>
+          <t>J1,J3,J4,J5</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Mini snap-action microswitch, hinge/roller lever (SPDT)</t>
+          <t>2-pin 2.54mm header</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>4x10-pack</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Amazon B0C6ZNBFDH</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="G18" s="8" t="n">
-        <v>31.96</v>
+        <v>3</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>31.96</v>
+        <v>3</v>
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
@@ -1208,44 +1208,44 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>lever pokes up through the playfield slot, the coin trips it (28 inputs; the 7 gobble switches parallel onto S23). Authentic alt: the Bally rollover-wire leaf switch is DISCONTINUED - Action Pinball SW-1A-120 ($8.39 ea, in stock) needs a rollover wireform. Reuse your originals if you have them.</t>
+          <t>power in + solenoid out</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Playfield</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>LED strip</t>
+          <t>Score / gobble switches</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>WS2812b 150-pixel 5V strip</t>
+          <t>Mini snap-action microswitch, hinge/roller lever (SPDT)</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>4x10-pack</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Amazon B0CFTPT81S</t>
+          <t>Amazon B0C6ZNBFDH</t>
         </is>
       </c>
       <c r="G19" s="12" t="n">
-        <v>12.99</v>
+        <v>31.96</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>12.99</v>
+        <v>31.96</v>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>150 addressable px</t>
+          <t>lever pokes up through the playfield slot, the coin trips it (28 inputs; the 7 gobble switches parallel onto S23). Authentic alt: the Bally rollover-wire leaf switch is DISCONTINUED - Action Pinball SW-1A-120 ($8.39 ea, in stock) needs a rollover wireform. Reuse your originals if you have them.</t>
         </is>
       </c>
     </row>
@@ -1266,32 +1266,32 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Score lamps</t>
+          <t>LED strip</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>#555 T10 wedge LED, 6.3V non-polar (frosted)</t>
+          <t>WS2812b 150-pixel 5V strip</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>25-pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Amazon (Keiurot)</t>
+          <t>Amazon B0CFTPT81S</t>
         </is>
       </c>
       <c r="G20" s="8" t="n">
-        <v>18</v>
+        <v>12.99</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>18</v>
+        <v>12.99</v>
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>16 lamps + a 2nd bulb on 100/200/300/400 (double bright) = 20; non-polar &amp; pre-resistored, runs safely under-driven on the 5V rail (board R = 0 ohm links)</t>
+          <t>150 addressable px</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1312,12 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Lamp sockets</t>
+          <t>Score lamps</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>T10/#555 wedge socket, pigtail leads</t>
+          <t>#555 T10 wedge LED, 6.3V non-polar (frosted)</t>
         </is>
       </c>
       <c r="D21" s="10" t="n">
@@ -1330,14 +1330,14 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Amazon B00VDOPPDE</t>
+          <t>Amazon (Keiurot)</t>
         </is>
       </c>
       <c r="G21" s="12" t="n">
-        <v>11.99</v>
+        <v>18</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>11.99</v>
+        <v>18</v>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
@@ -1346,132 +1346,132 @@
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>one per bulb; solder its leads to the J2 lamp lines</t>
+          <t>16 lamps + a 2nd bulb on 100/200/300/400 (double bright) = 20; non-polar &amp; pre-resistored, runs safely under-driven on the 5V rail (board R = 0 ohm links)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Lamp sockets</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>T10/#555 wedge socket, pigtail leads</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>25-pack</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Amazon B00VDOPPDE</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>one per bulb; solder its leads to the J2 lamp lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
           <t>Actuators</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Coin-Lock, Win-Lock</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>SparkFun Solenoid - 5V (Small)</t>
         </is>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D23" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>each</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>SparkFun ROB-11015</t>
         </is>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G23" s="12" t="n">
         <v>4.95</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H23" s="12" t="n">
         <v>9.9</v>
       </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>small 5 V coils, ~4.5 mm throw</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Computer</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>mini-PC</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>PELADN Ryzen 5 5600H, 16GB DDR4 / 512GB SSD</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Amazon B0F7R7V9VK</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="n">
-        <v>209.99</v>
-      </c>
-      <c r="H24" s="8" t="n">
-        <v>209.99</v>
-      </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>6C/12T Ryzen, Vega gfx, WiFi6, USB3.2 — plenty of headroom</t>
-        </is>
-      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="n"/>
+      <c r="J24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Display</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>monitor</t>
+          <t>mini-PC</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>QQU 15.6" portable touchscreen (with stand)</t>
+          <t>PELADN Ryzen 5 5600H, 16GB DDR4 / 512GB SSD</t>
         </is>
       </c>
       <c r="D25" s="10" t="n">
@@ -1484,14 +1484,14 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Amazon B0FHHM1Y7Z</t>
+          <t>Amazon B0F7R7V9VK</t>
         </is>
       </c>
       <c r="G25" s="12" t="n">
-        <v>70.48999999999999</v>
+        <v>209.99</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>70.48999999999999</v>
+        <v>209.99</v>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
@@ -1500,24 +1500,24 @@
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>1080P IPS/HDR; USB-C touch + HDMI; incl. stand</t>
+          <t>6C/12T Ryzen, Vega gfx, WiFi6, USB3.2 — plenty of headroom</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>Display</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>monitor</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>4-port USB 2.0 hub</t>
+          <t>QQU 15.6" portable touchscreen (with stand)</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
@@ -1530,14 +1530,14 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Amazon/Monoprice</t>
+          <t>Amazon B0FHHM1Y7Z</t>
         </is>
       </c>
       <c r="G26" s="8" t="n">
-        <v>8.99</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>8.99</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
@@ -1546,24 +1546,24 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>one port per FT232H</t>
+          <t>1080P IPS/HDR; USB-C touch + HDMI; incl. stand</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>J1 supply</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>3.3 V DC wall adapter (≥1A)</t>
+          <t>4-port USB 2.0 hub</t>
         </is>
       </c>
       <c r="D27" s="10" t="n">
@@ -1576,14 +1576,14 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Amazon B07BGW2VXV</t>
+          <t>Amazon/Monoprice</t>
         </is>
       </c>
       <c r="G27" s="12" t="n">
-        <v>7.99</v>
+        <v>8.99</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>7.99</v>
+        <v>8.99</v>
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>switch-common / GPIO logic</t>
+          <t>one port per FT232H</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>J3 / LED± supply</t>
+          <t>J1 supply</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>5 V DC wall adapter (≥5A)</t>
+          <t>3.3 V DC wall adapter (≥1A)</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
@@ -1622,39 +1622,85 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
+          <t>Amazon B07BGW2VXV</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>switch-common / GPIO logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>J3 / LED± supply</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>5 V DC wall adapter (≥5A)</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
           <t>Amazon (5V 5A)</t>
         </is>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G29" s="12" t="n">
         <v>12.99</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H29" s="12" t="n">
         <v>12.99</v>
       </c>
-      <c r="I28" s="9" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
         <is>
           <t>size for LED strip + lamps + coils</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="G30" s="14" t="inlineStr">
+    <row r="31">
+      <c r="G31" s="14" t="inlineStr">
         <is>
           <t>ESTIMATED TOTAL</t>
         </is>
       </c>
-      <c r="H30" s="15">
-        <f>SUM(H5:H28)</f>
+      <c r="H31" s="15">
+        <f>SUM(H5:H29)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="C31" s="16" t="inlineStr">
+    <row r="32">
+      <c r="C32" s="16" t="inlineStr">
         <is>
           <t>Line est already accounts for quantity (e.g. 4× FT232H). Pack/kit rows are a single purchase that covers the qty.</t>
         </is>
@@ -1662,9 +1708,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A24:J24"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <hyperlinks>
@@ -1685,11 +1731,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Switches: spec the arcade coin switch (85mm wire actuator)
The right part is a coin switch - a snap-action microswitch with a long
thin wire actuator (like the Bally original). The wire pokes up through a
playfield slot and the rolling coin trips it; the long wire = feather-light
force. Mounts hidden under the playfield, wires like any SPDT switch (no
board changes). $3.99 ea (DIY Retro Arcade), ~$2 in 10-packs. Updated the
BOM, guide, README and redrew the switch glyph to match. BOM now $610.86.
</commit_message>
<xml_diff>
--- a/docs/SkillGame BOM (sourced).xlsx
+++ b/docs/SkillGame BOM (sourced).xlsx
@@ -1225,7 +1225,7 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Mini snap-action microswitch, hinge/roller lever (SPDT)</t>
+          <t>Arcade COIN SWITCH, 85mm straight wire actuator (SPDT)</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
@@ -1233,19 +1233,19 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>4x10-pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Amazon B0C6ZNBFDH</t>
+          <t>DIY Retro Arcade / eBay</t>
         </is>
       </c>
       <c r="G19" s="12" t="n">
-        <v>31.96</v>
+        <v>3.99</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>31.96</v>
+        <v>135.66</v>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>lever pokes up through the playfield slot, the coin trips it (28 inputs; the 7 gobble switches parallel onto S23). Authentic alt: the Bally rollover-wire leaf switch is DISCONTINUED - Action Pinball SW-1A-120 ($8.39 ea, in stock) needs a rollover wireform. Reuse your originals if you have them.</t>
+          <t>the long wire pokes up through a playfield slot; the rolling coin trips it (the 85mm wire = tiny actuation force, made for coins). Mounts hidden UNDER the playfield. Wires like any SPDT switch (use COM + NO). 28 inputs; the 7 gobble switches parallel onto S23. ~$2 ea in 10-packs on eBay/AliExpress.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Solenoids: pulse the spring-return locks, never hold them energized
The Win-Lock and Coin-Lock are spring-return coils (plunger out at rest
blocks a coin with no power; a pulse retracts it to drop the coin). The
old Winner() held the Win-Lock on for the rest of the game, which would
cook the intermittent-duty coil.

- Winner() now lights the LEDs only; the winning coin is held by the
  spring, and released by a pulse on the next coin-up.
- Coin-up pulses the Coin-Lock to drop the inserted coin onto the rails,
  and releases any held winner coin. Real play only, never in demo.
- New ILampSink.PulseSolenoid; +4 tests (56 total).
- Schematic page, README, assembly guide and BOM note the mechanism.
</commit_message>
<xml_diff>
--- a/docs/SkillGame BOM (sourced).xlsx
+++ b/docs/SkillGame BOM (sourced).xlsx
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>SparkFun Solenoid - 5V (Small)</t>
+          <t>SparkFun Solenoid - 5V (Small), ROB-11015</t>
         </is>
       </c>
       <c r="D23" s="10" t="n">
@@ -1426,10 +1426,10 @@
         </is>
       </c>
       <c r="G23" s="12" t="n">
-        <v>4.95</v>
+        <v>6.5</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>9.9</v>
+        <v>13</v>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>small 5 V coils, ~4.5 mm throw</t>
+          <t>5 V, 1.1 A, 4.5 ohm, ~5.5 W. SPRING-RETURN push-pull: plunger sits OUT at rest (blocks a coin, zero power) and retracts when energized (drops it). INTERMITTENT duty (25%) - the firmware PULSES it, never holds. T2A fuse each (F1/F2). Same part as Adafruit 2776.</t>
         </is>
       </c>
     </row>

</xml_diff>